<commit_message>
better stats and fed math battles
</commit_message>
<xml_diff>
--- a/Austerlitz/Turns/136HJan1808a.xlsx
+++ b/Austerlitz/Turns/136HJan1808a.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\Austerlitz\Austerlitz\Turns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7643EB3A-132E-45FE-9B0E-FCCAE1CDBA74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C0D554F-19DD-4F14-AA3A-8B4E2245CCFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7671,7 +7671,7 @@
         <v>4156</v>
       </c>
       <c r="C215" s="11">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D215" s="11">
         <v>1</v>

</xml_diff>

<commit_message>
lots of boarding chamgoes and refactor
</commit_message>
<xml_diff>
--- a/Austerlitz/Turns/136HJan1808a.xlsx
+++ b/Austerlitz/Turns/136HJan1808a.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\Austerlitz\Austerlitz\Turns\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B252632-842A-431E-9A67-59B3760B06D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{070522E1-DC5C-4FC9-AE24-A206B9D7F39F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="1530" windowWidth="18060" windowHeight="20070" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27345" yWindow="2190" windowWidth="18060" windowHeight="20070" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -529,7 +529,31 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="5">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF4C7C3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF4C7C3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor auto="1"/>
+          <bgColor rgb="FFF4C7C3"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1037,17 +1061,19 @@
       <c r="C13" s="11">
         <v>206</v>
       </c>
-      <c r="D13" s="11">
-        <v>4720000</v>
+      <c r="D13" s="12">
+        <v>5352000</v>
       </c>
       <c r="E13" s="11">
         <v>32000</v>
       </c>
       <c r="F13" s="11">
-        <v>7488</v>
+        <v>6624</v>
       </c>
       <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
+      <c r="H13" s="11">
+        <v>5600</v>
+      </c>
       <c r="I13" s="11"/>
       <c r="K13" s="6"/>
       <c r="L13" s="6" t="str">
@@ -1466,16 +1492,16 @@
         <v>1</v>
       </c>
       <c r="D34" s="11">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="E34" s="11">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F34" s="11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G34" s="11">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="H34" s="11"/>
       <c r="I34" s="11"/>
@@ -1515,16 +1541,16 @@
         <v>1</v>
       </c>
       <c r="D35" s="11">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="E35" s="11">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F35" s="11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G35" s="11">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="H35" s="11"/>
       <c r="I35" s="11"/>
@@ -1551,13 +1577,13 @@
         <v>1</v>
       </c>
       <c r="E36" s="11">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F36" s="11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G36" s="11">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="H36" s="11"/>
       <c r="I36" s="11"/>
@@ -1584,13 +1610,13 @@
         <v>1</v>
       </c>
       <c r="E37" s="11">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F37" s="11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G37" s="11">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="H37" s="11"/>
       <c r="I37" s="11"/>
@@ -1617,13 +1643,13 @@
         <v>1</v>
       </c>
       <c r="E38" s="11">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F38" s="11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G38" s="11">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="H38" s="11"/>
       <c r="I38" s="11"/>
@@ -1650,13 +1676,13 @@
         <v>1</v>
       </c>
       <c r="E39" s="11">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F39" s="11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G39" s="11">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="H39" s="11"/>
       <c r="I39" s="11"/>
@@ -1677,19 +1703,19 @@
         <v>206</v>
       </c>
       <c r="C40" s="11">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="D40" s="11">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="E40" s="11">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F40" s="11">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G40" s="11">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="H40" s="11"/>
       <c r="I40" s="11"/>
@@ -1716,13 +1742,13 @@
         <v>19</v>
       </c>
       <c r="E41" s="11">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="F41" s="11">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="G41" s="11">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="H41" s="11"/>
       <c r="I41" s="11"/>
@@ -3702,8 +3728,12 @@
       <c r="A133" s="5">
         <v>1</v>
       </c>
-      <c r="B133" s="11"/>
-      <c r="C133" s="11"/>
+      <c r="B133" s="11">
+        <v>76</v>
+      </c>
+      <c r="C133" s="11">
+        <v>96</v>
+      </c>
       <c r="D133" s="5"/>
       <c r="E133" s="5"/>
       <c r="F133" s="5"/>
@@ -4356,13 +4386,13 @@
         <v>8</v>
       </c>
       <c r="B150" s="11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C150" s="11">
         <v>29</v>
       </c>
       <c r="D150" s="11">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E150" s="5"/>
       <c r="F150" s="21"/>
@@ -4403,13 +4433,13 @@
         <v>9</v>
       </c>
       <c r="B151" s="11">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C151" s="11">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="D151" s="11">
-        <v>27</v>
+        <v>96</v>
       </c>
       <c r="E151" s="5"/>
       <c r="F151" s="21"/>
@@ -13081,14 +13111,29 @@
     <mergeCell ref="G5:I5"/>
     <mergeCell ref="G6:I6"/>
   </mergeCells>
+  <conditionalFormatting sqref="B25:C30 B45:C50 B54:C65 B69:B84 B88:E91 B95:E102 B106:B111 B115:F122 B126:B129 B133:C139 B143:D152 B156:C176 B180:C184 B188:G190 B194:E211 B248:E265 B269:E284 B288:C293 B297:H300 B304:C307">
+    <cfRule type="expression" dxfId="4" priority="6">
+      <formula>AND($L25 &lt;&gt; "Valid",$L25&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B215:H244">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>AND($L215 &lt;&gt; "Valid",$L215&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B12:I21 B25:C30 B34:J41 B45:C50 B54:C65 B69:B84 B88:E91 B95:E102 B106:B111 B115:F122 B126:B129 B133:C139 B143:D152 B156:C176 B180:C184 B188:G190 B194:E211 B248:E265 B269:E284 B288:C293 B297:H300 B304:C307">
-    <cfRule type="expression" dxfId="0" priority="3">
+  <conditionalFormatting sqref="B12:I12 B14:I21 I13">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>AND($L12 &lt;&gt; "Valid",$L12&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B13:H13">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>AND($L13 &lt;&gt; "Valid",$L13&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B34:J41">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND($L34 &lt;&gt; "Valid",$L34&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">

</xml_diff>